<commit_message>
final changes to repo file
</commit_message>
<xml_diff>
--- a/data/temp/Indian_Repo_Rate_Data.xlsx
+++ b/data/temp/Indian_Repo_Rate_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Spandan Dutta\econometrics_project\data\temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56D70365-F516-40A2-8992-E7B5CE1F7A42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7763F57B-567C-4F5E-8E54-8710FC05E1D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="156" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -414,8 +414,8 @@
         <v>8</v>
       </c>
       <c r="D4" s="1">
-        <f>0.049 * $F$2</f>
-        <v>0</v>
+        <f>0.049 * 100</f>
+        <v>4.9000000000000004</v>
       </c>
       <c r="E4" s="1"/>
     </row>

</xml_diff>

<commit_message>
cleaned repo rate data
</commit_message>
<xml_diff>
--- a/data/temp/Indian_Repo_Rate_Data.xlsx
+++ b/data/temp/Indian_Repo_Rate_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Spandan Dutta\econometrics_project\data\temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7763F57B-567C-4F5E-8E54-8710FC05E1D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A34093C-1180-4D34-8C85-B617BD5362B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="156" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,9 +35,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="17">
   <si>
-    <t>Your Dictionary Date</t>
-  </si>
-  <si>
     <t>Exact RBI Announcement Date</t>
   </si>
   <si>
@@ -84,6 +81,9 @@
   </si>
   <si>
     <t>2025-04-30'</t>
+  </si>
+  <si>
+    <t>Dictionary Date</t>
   </si>
 </sst>
 </file>
@@ -359,28 +359,28 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
       </c>
       <c r="E1" s="1"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>6</v>
       </c>
       <c r="D2" s="1">
         <v>4</v>
@@ -389,13 +389,13 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" s="3">
         <v>44685</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D3" s="1">
         <f>0.044*100</f>
@@ -405,13 +405,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" s="3">
         <v>44720</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D4" s="1">
         <f>0.049 * 100</f>
@@ -421,13 +421,13 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5" s="3">
         <v>44778</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5" s="1">
         <f>0.054*100</f>
@@ -437,13 +437,13 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" s="3">
         <v>44834</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D6" s="1">
         <f>0.059*100</f>
@@ -453,13 +453,13 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B7" s="3">
         <v>44902</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D7" s="1">
         <f>0.0625*100</f>
@@ -469,13 +469,13 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" s="3">
         <v>44965</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D8" s="1">
         <f>0.065*100</f>
@@ -485,13 +485,13 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B9" s="3">
         <v>45695</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D9" s="1">
         <f>0.0625*100</f>
@@ -501,13 +501,13 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B10" s="3">
         <v>45756</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D10" s="1">
         <f>0.06*100</f>

</xml_diff>